<commit_message>
feat: Major updates across 5 components
- Updated 1 lambda function files
- Modified 1 frontend files
- Updated 2 configuration files
- Enhanced 1 core system files
- Modified 1 test files
- Total files changed: 6
-  6 files changed, 353 insertions(+), 152 deletions(-)

[AUTOMATED] Generated with [Claude Code](https://claude.ai/code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/test_cases/financial_portfolio/20250701_161107/extracted_results/original_files/financial_portfolio.xlsx
+++ b/tests/test_cases/financial_portfolio/20250701_161107/extracted_results/original_files/financial_portfolio.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eliyahuai-my.sharepoint.com/personal/eliyahu_eliyahu_ai/Documents/Desktop/src/perplexityValidator/tests/test_cases/financial_portfolio/20250701_161107/extracted_results/original_files/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_75ED61FAF613C8264F2C4CDC55D1AF60449CBEEB" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A33D86CC-3E63-4A39-B163-2C5A3D7EC77D}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>Ticker_Symbol</t>
   </si>
@@ -146,13 +152,22 @@
   </si>
   <si>
     <t>2024-12-15</t>
+  </si>
+  <si>
+    <t>Latest News</t>
+  </si>
+  <si>
+    <t>Projections</t>
+  </si>
+  <si>
+    <t>Invest Now?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -177,7 +192,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -200,13 +215,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -215,13 +244,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -259,7 +296,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -293,6 +330,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -327,9 +365,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -502,11 +541,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="24.1796875" customWidth="1"/>
+    <col min="4" max="4" width="15.453125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -531,8 +574,17 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -558,7 +610,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -584,7 +636,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -598,7 +650,7 @@
         <v>39</v>
       </c>
       <c r="E4">
-        <v>153.92</v>
+        <v>153.91999999999999</v>
       </c>
       <c r="F4">
         <v>1598.4</v>
@@ -610,7 +662,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -636,7 +688,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>12</v>
       </c>
@@ -662,7 +714,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -688,7 +740,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>14</v>
       </c>
@@ -702,10 +754,10 @@
         <v>41</v>
       </c>
       <c r="E8">
-        <v>72.18000000000001</v>
+        <v>72.180000000000007</v>
       </c>
       <c r="F8">
-        <v>573.2</v>
+        <v>573.20000000000005</v>
       </c>
       <c r="G8">
         <v>26.9</v>
@@ -714,7 +766,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -740,7 +792,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -757,7 +809,7 @@
         <v>166.12</v>
       </c>
       <c r="F10">
-        <v>2067.8</v>
+        <v>2067.8000000000002</v>
       </c>
       <c r="G10">
         <v>26.4</v>
@@ -766,7 +818,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>17</v>
       </c>

</xml_diff>